<commit_message>
Switch attendance punching to PC via Microsoft Forms
Staff submit a pre-filled Forms link that opens at Windows sign-in; a
Forms-triggered flow records server time to the admin's private Excel
and Outlook calendar. Drops phone location columns from the template.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GSEq5iGzfmWaXkgHVFes9g
</commit_message>
<xml_diff>
--- a/kintai/power-automate/勤怠記録.xlsx
+++ b/kintai/power-automate/勤怠記録.xlsx
@@ -85,10 +85,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -99,7 +99,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -190,9 +189,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="打刻" displayName="打刻" ref="A1:O2" headerRowCount="1">
-  <autoFilter ref="A1:O2"/>
-  <tableColumns count="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="打刻" displayName="打刻" ref="A1:K2" headerRowCount="1">
+  <autoFilter ref="A1:K2"/>
+  <tableColumns count="11">
     <tableColumn id="1" name="Key"/>
     <tableColumn id="2" name="日付"/>
     <tableColumn id="3" name="時刻"/>
@@ -202,12 +201,8 @@
     <tableColumn id="7" name="種類"/>
     <tableColumn id="8" name="初回"/>
     <tableColumn id="9" name="遅刻分"/>
-    <tableColumn id="10" name="場所"/>
-    <tableColumn id="11" name="緯度"/>
-    <tableColumn id="12" name="経度"/>
-    <tableColumn id="13" name="住所"/>
-    <tableColumn id="14" name="記録日時"/>
-    <tableColumn id="15" name="備考"/>
+    <tableColumn id="10" name="記録日時"/>
+    <tableColumn id="11" name="備考"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -502,16 +497,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -527,7 +521,7 @@
           <t>集計する月（例：202610 ＝ 2026年10月）</t>
         </is>
       </c>
-      <c r="B3" s="9" t="n">
+      <c r="B3" s="2" t="n">
         <v>202610</v>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -563,11 +557,6 @@
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>社外・不明の打刻</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>メモ</t>
         </is>
@@ -580,22 +569,18 @@
         <v/>
       </c>
       <c r="C6" s="7">
-        <f>IF($A6="","",COUNTIFS(打刻!F:F,$A6,打刻!D:D,$B$3,打刻!H:H,"○"))</f>
+        <f>IF($A6="","",COUNTIFS(打刻!F:F,$A6,打刻!D:D,$B$3,打刻!G:G,"出勤",打刻!H:H,"○"))</f>
         <v/>
       </c>
       <c r="D6" s="7">
-        <f>IF($A6="","",COUNTIFS(打刻!F:F,$A6,打刻!D:D,$B$3,打刻!H:H,"○",打刻!I:I,"&gt;0"))</f>
+        <f>IF($A6="","",COUNTIFS(打刻!F:F,$A6,打刻!D:D,$B$3,打刻!G:G,"出勤",打刻!H:H,"○",打刻!I:I,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E6" s="7">
-        <f>IF($A6="","",SUMIFS(打刻!I:I,打刻!F:F,$A6,打刻!D:D,$B$3,打刻!H:H,"○"))</f>
-        <v/>
-      </c>
-      <c r="F6" s="7">
-        <f>IF($A6="","",COUNTIFS(打刻!F:F,$A6,打刻!D:D,$B$3,打刻!J:J,"社外")+COUNTIFS(打刻!F:F,$A6,打刻!D:D,$B$3,打刻!J:J,"不明"))</f>
-        <v/>
-      </c>
-      <c r="G6" s="6" t="n"/>
+        <f>IF($A6="","",SUMIFS(打刻!I:I,打刻!F:F,$A6,打刻!D:D,$B$3,打刻!G:G,"出勤",打刻!H:H,"○"))</f>
+        <v/>
+      </c>
+      <c r="F6" s="6" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n"/>
@@ -604,22 +589,18 @@
         <v/>
       </c>
       <c r="C7" s="7">
-        <f>IF($A7="","",COUNTIFS(打刻!F:F,$A7,打刻!D:D,$B$3,打刻!H:H,"○"))</f>
+        <f>IF($A7="","",COUNTIFS(打刻!F:F,$A7,打刻!D:D,$B$3,打刻!G:G,"出勤",打刻!H:H,"○"))</f>
         <v/>
       </c>
       <c r="D7" s="7">
-        <f>IF($A7="","",COUNTIFS(打刻!F:F,$A7,打刻!D:D,$B$3,打刻!H:H,"○",打刻!I:I,"&gt;0"))</f>
+        <f>IF($A7="","",COUNTIFS(打刻!F:F,$A7,打刻!D:D,$B$3,打刻!G:G,"出勤",打刻!H:H,"○",打刻!I:I,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E7" s="7">
-        <f>IF($A7="","",SUMIFS(打刻!I:I,打刻!F:F,$A7,打刻!D:D,$B$3,打刻!H:H,"○"))</f>
-        <v/>
-      </c>
-      <c r="F7" s="7">
-        <f>IF($A7="","",COUNTIFS(打刻!F:F,$A7,打刻!D:D,$B$3,打刻!J:J,"社外")+COUNTIFS(打刻!F:F,$A7,打刻!D:D,$B$3,打刻!J:J,"不明"))</f>
-        <v/>
-      </c>
-      <c r="G7" s="6" t="n"/>
+        <f>IF($A7="","",SUMIFS(打刻!I:I,打刻!F:F,$A7,打刻!D:D,$B$3,打刻!G:G,"出勤",打刻!H:H,"○"))</f>
+        <v/>
+      </c>
+      <c r="F7" s="6" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="n"/>
@@ -628,22 +609,18 @@
         <v/>
       </c>
       <c r="C8" s="7">
-        <f>IF($A8="","",COUNTIFS(打刻!F:F,$A8,打刻!D:D,$B$3,打刻!H:H,"○"))</f>
+        <f>IF($A8="","",COUNTIFS(打刻!F:F,$A8,打刻!D:D,$B$3,打刻!G:G,"出勤",打刻!H:H,"○"))</f>
         <v/>
       </c>
       <c r="D8" s="7">
-        <f>IF($A8="","",COUNTIFS(打刻!F:F,$A8,打刻!D:D,$B$3,打刻!H:H,"○",打刻!I:I,"&gt;0"))</f>
+        <f>IF($A8="","",COUNTIFS(打刻!F:F,$A8,打刻!D:D,$B$3,打刻!G:G,"出勤",打刻!H:H,"○",打刻!I:I,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E8" s="7">
-        <f>IF($A8="","",SUMIFS(打刻!I:I,打刻!F:F,$A8,打刻!D:D,$B$3,打刻!H:H,"○"))</f>
-        <v/>
-      </c>
-      <c r="F8" s="7">
-        <f>IF($A8="","",COUNTIFS(打刻!F:F,$A8,打刻!D:D,$B$3,打刻!J:J,"社外")+COUNTIFS(打刻!F:F,$A8,打刻!D:D,$B$3,打刻!J:J,"不明"))</f>
-        <v/>
-      </c>
-      <c r="G8" s="6" t="n"/>
+        <f>IF($A8="","",SUMIFS(打刻!I:I,打刻!F:F,$A8,打刻!D:D,$B$3,打刻!G:G,"出勤",打刻!H:H,"○"))</f>
+        <v/>
+      </c>
+      <c r="F8" s="6" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n"/>
@@ -652,22 +629,18 @@
         <v/>
       </c>
       <c r="C9" s="7">
-        <f>IF($A9="","",COUNTIFS(打刻!F:F,$A9,打刻!D:D,$B$3,打刻!H:H,"○"))</f>
+        <f>IF($A9="","",COUNTIFS(打刻!F:F,$A9,打刻!D:D,$B$3,打刻!G:G,"出勤",打刻!H:H,"○"))</f>
         <v/>
       </c>
       <c r="D9" s="7">
-        <f>IF($A9="","",COUNTIFS(打刻!F:F,$A9,打刻!D:D,$B$3,打刻!H:H,"○",打刻!I:I,"&gt;0"))</f>
+        <f>IF($A9="","",COUNTIFS(打刻!F:F,$A9,打刻!D:D,$B$3,打刻!G:G,"出勤",打刻!H:H,"○",打刻!I:I,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E9" s="7">
-        <f>IF($A9="","",SUMIFS(打刻!I:I,打刻!F:F,$A9,打刻!D:D,$B$3,打刻!H:H,"○"))</f>
-        <v/>
-      </c>
-      <c r="F9" s="7">
-        <f>IF($A9="","",COUNTIFS(打刻!F:F,$A9,打刻!D:D,$B$3,打刻!J:J,"社外")+COUNTIFS(打刻!F:F,$A9,打刻!D:D,$B$3,打刻!J:J,"不明"))</f>
-        <v/>
-      </c>
-      <c r="G9" s="6" t="n"/>
+        <f>IF($A9="","",SUMIFS(打刻!I:I,打刻!F:F,$A9,打刻!D:D,$B$3,打刻!G:G,"出勤",打刻!H:H,"○"))</f>
+        <v/>
+      </c>
+      <c r="F9" s="6" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="n"/>
@@ -676,22 +649,18 @@
         <v/>
       </c>
       <c r="C10" s="7">
-        <f>IF($A10="","",COUNTIFS(打刻!F:F,$A10,打刻!D:D,$B$3,打刻!H:H,"○"))</f>
+        <f>IF($A10="","",COUNTIFS(打刻!F:F,$A10,打刻!D:D,$B$3,打刻!G:G,"出勤",打刻!H:H,"○"))</f>
         <v/>
       </c>
       <c r="D10" s="7">
-        <f>IF($A10="","",COUNTIFS(打刻!F:F,$A10,打刻!D:D,$B$3,打刻!H:H,"○",打刻!I:I,"&gt;0"))</f>
+        <f>IF($A10="","",COUNTIFS(打刻!F:F,$A10,打刻!D:D,$B$3,打刻!G:G,"出勤",打刻!H:H,"○",打刻!I:I,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E10" s="7">
-        <f>IF($A10="","",SUMIFS(打刻!I:I,打刻!F:F,$A10,打刻!D:D,$B$3,打刻!H:H,"○"))</f>
-        <v/>
-      </c>
-      <c r="F10" s="7">
-        <f>IF($A10="","",COUNTIFS(打刻!F:F,$A10,打刻!D:D,$B$3,打刻!J:J,"社外")+COUNTIFS(打刻!F:F,$A10,打刻!D:D,$B$3,打刻!J:J,"不明"))</f>
-        <v/>
-      </c>
-      <c r="G10" s="6" t="n"/>
+        <f>IF($A10="","",SUMIFS(打刻!I:I,打刻!F:F,$A10,打刻!D:D,$B$3,打刻!G:G,"出勤",打刻!H:H,"○"))</f>
+        <v/>
+      </c>
+      <c r="F10" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n"/>
@@ -700,22 +669,18 @@
         <v/>
       </c>
       <c r="C11" s="7">
-        <f>IF($A11="","",COUNTIFS(打刻!F:F,$A11,打刻!D:D,$B$3,打刻!H:H,"○"))</f>
+        <f>IF($A11="","",COUNTIFS(打刻!F:F,$A11,打刻!D:D,$B$3,打刻!G:G,"出勤",打刻!H:H,"○"))</f>
         <v/>
       </c>
       <c r="D11" s="7">
-        <f>IF($A11="","",COUNTIFS(打刻!F:F,$A11,打刻!D:D,$B$3,打刻!H:H,"○",打刻!I:I,"&gt;0"))</f>
+        <f>IF($A11="","",COUNTIFS(打刻!F:F,$A11,打刻!D:D,$B$3,打刻!G:G,"出勤",打刻!H:H,"○",打刻!I:I,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E11" s="7">
-        <f>IF($A11="","",SUMIFS(打刻!I:I,打刻!F:F,$A11,打刻!D:D,$B$3,打刻!H:H,"○"))</f>
-        <v/>
-      </c>
-      <c r="F11" s="7">
-        <f>IF($A11="","",COUNTIFS(打刻!F:F,$A11,打刻!D:D,$B$3,打刻!J:J,"社外")+COUNTIFS(打刻!F:F,$A11,打刻!D:D,$B$3,打刻!J:J,"不明"))</f>
-        <v/>
-      </c>
-      <c r="G11" s="6" t="n"/>
+        <f>IF($A11="","",SUMIFS(打刻!I:I,打刻!F:F,$A11,打刻!D:D,$B$3,打刻!G:G,"出勤",打刻!H:H,"○"))</f>
+        <v/>
+      </c>
+      <c r="F11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="n"/>
@@ -724,22 +689,18 @@
         <v/>
       </c>
       <c r="C12" s="7">
-        <f>IF($A12="","",COUNTIFS(打刻!F:F,$A12,打刻!D:D,$B$3,打刻!H:H,"○"))</f>
+        <f>IF($A12="","",COUNTIFS(打刻!F:F,$A12,打刻!D:D,$B$3,打刻!G:G,"出勤",打刻!H:H,"○"))</f>
         <v/>
       </c>
       <c r="D12" s="7">
-        <f>IF($A12="","",COUNTIFS(打刻!F:F,$A12,打刻!D:D,$B$3,打刻!H:H,"○",打刻!I:I,"&gt;0"))</f>
+        <f>IF($A12="","",COUNTIFS(打刻!F:F,$A12,打刻!D:D,$B$3,打刻!G:G,"出勤",打刻!H:H,"○",打刻!I:I,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E12" s="7">
-        <f>IF($A12="","",SUMIFS(打刻!I:I,打刻!F:F,$A12,打刻!D:D,$B$3,打刻!H:H,"○"))</f>
-        <v/>
-      </c>
-      <c r="F12" s="7">
-        <f>IF($A12="","",COUNTIFS(打刻!F:F,$A12,打刻!D:D,$B$3,打刻!J:J,"社外")+COUNTIFS(打刻!F:F,$A12,打刻!D:D,$B$3,打刻!J:J,"不明"))</f>
-        <v/>
-      </c>
-      <c r="G12" s="6" t="n"/>
+        <f>IF($A12="","",SUMIFS(打刻!I:I,打刻!F:F,$A12,打刻!D:D,$B$3,打刻!G:G,"出勤",打刻!H:H,"○"))</f>
+        <v/>
+      </c>
+      <c r="F12" s="6" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n"/>
@@ -748,22 +709,18 @@
         <v/>
       </c>
       <c r="C13" s="7">
-        <f>IF($A13="","",COUNTIFS(打刻!F:F,$A13,打刻!D:D,$B$3,打刻!H:H,"○"))</f>
+        <f>IF($A13="","",COUNTIFS(打刻!F:F,$A13,打刻!D:D,$B$3,打刻!G:G,"出勤",打刻!H:H,"○"))</f>
         <v/>
       </c>
       <c r="D13" s="7">
-        <f>IF($A13="","",COUNTIFS(打刻!F:F,$A13,打刻!D:D,$B$3,打刻!H:H,"○",打刻!I:I,"&gt;0"))</f>
+        <f>IF($A13="","",COUNTIFS(打刻!F:F,$A13,打刻!D:D,$B$3,打刻!G:G,"出勤",打刻!H:H,"○",打刻!I:I,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E13" s="7">
-        <f>IF($A13="","",SUMIFS(打刻!I:I,打刻!F:F,$A13,打刻!D:D,$B$3,打刻!H:H,"○"))</f>
-        <v/>
-      </c>
-      <c r="F13" s="7">
-        <f>IF($A13="","",COUNTIFS(打刻!F:F,$A13,打刻!D:D,$B$3,打刻!J:J,"社外")+COUNTIFS(打刻!F:F,$A13,打刻!D:D,$B$3,打刻!J:J,"不明"))</f>
-        <v/>
-      </c>
-      <c r="G13" s="6" t="n"/>
+        <f>IF($A13="","",SUMIFS(打刻!I:I,打刻!F:F,$A13,打刻!D:D,$B$3,打刻!G:G,"出勤",打刻!H:H,"○"))</f>
+        <v/>
+      </c>
+      <c r="F13" s="6" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="n"/>
@@ -772,22 +729,18 @@
         <v/>
       </c>
       <c r="C14" s="7">
-        <f>IF($A14="","",COUNTIFS(打刻!F:F,$A14,打刻!D:D,$B$3,打刻!H:H,"○"))</f>
+        <f>IF($A14="","",COUNTIFS(打刻!F:F,$A14,打刻!D:D,$B$3,打刻!G:G,"出勤",打刻!H:H,"○"))</f>
         <v/>
       </c>
       <c r="D14" s="7">
-        <f>IF($A14="","",COUNTIFS(打刻!F:F,$A14,打刻!D:D,$B$3,打刻!H:H,"○",打刻!I:I,"&gt;0"))</f>
+        <f>IF($A14="","",COUNTIFS(打刻!F:F,$A14,打刻!D:D,$B$3,打刻!G:G,"出勤",打刻!H:H,"○",打刻!I:I,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E14" s="7">
-        <f>IF($A14="","",SUMIFS(打刻!I:I,打刻!F:F,$A14,打刻!D:D,$B$3,打刻!H:H,"○"))</f>
-        <v/>
-      </c>
-      <c r="F14" s="7">
-        <f>IF($A14="","",COUNTIFS(打刻!F:F,$A14,打刻!D:D,$B$3,打刻!J:J,"社外")+COUNTIFS(打刻!F:F,$A14,打刻!D:D,$B$3,打刻!J:J,"不明"))</f>
-        <v/>
-      </c>
-      <c r="G14" s="6" t="n"/>
+        <f>IF($A14="","",SUMIFS(打刻!I:I,打刻!F:F,$A14,打刻!D:D,$B$3,打刻!G:G,"出勤",打刻!H:H,"○"))</f>
+        <v/>
+      </c>
+      <c r="F14" s="6" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="n"/>
@@ -796,52 +749,43 @@
         <v/>
       </c>
       <c r="C15" s="7">
-        <f>IF($A15="","",COUNTIFS(打刻!F:F,$A15,打刻!D:D,$B$3,打刻!H:H,"○"))</f>
+        <f>IF($A15="","",COUNTIFS(打刻!F:F,$A15,打刻!D:D,$B$3,打刻!G:G,"出勤",打刻!H:H,"○"))</f>
         <v/>
       </c>
       <c r="D15" s="7">
-        <f>IF($A15="","",COUNTIFS(打刻!F:F,$A15,打刻!D:D,$B$3,打刻!H:H,"○",打刻!I:I,"&gt;0"))</f>
+        <f>IF($A15="","",COUNTIFS(打刻!F:F,$A15,打刻!D:D,$B$3,打刻!G:G,"出勤",打刻!H:H,"○",打刻!I:I,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E15" s="7">
-        <f>IF($A15="","",SUMIFS(打刻!I:I,打刻!F:F,$A15,打刻!D:D,$B$3,打刻!H:H,"○"))</f>
-        <v/>
-      </c>
-      <c r="F15" s="7">
-        <f>IF($A15="","",COUNTIFS(打刻!F:F,$A15,打刻!D:D,$B$3,打刻!J:J,"社外")+COUNTIFS(打刻!F:F,$A15,打刻!D:D,$B$3,打刻!J:J,"不明"))</f>
-        <v/>
-      </c>
-      <c r="G15" s="6" t="n"/>
+        <f>IF($A15="","",SUMIFS(打刻!I:I,打刻!F:F,$A15,打刻!D:D,$B$3,打刻!G:G,"出勤",打刻!H:H,"○"))</f>
+        <v/>
+      </c>
+      <c r="F15" s="6" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>・出勤日数／遅刻は、その日の最初の「出勤」打刻で判定します（2回押しても二重には数えません）。</t>
+          <t>・出勤日数／遅刻は、その日の最初の「出勤」で判定します（2回送っても二重には数えません）。</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>・「社外」は会社から離れた場所での打刻、「不明」はスマホ以外（PCなど）で位置情報が無い打刻です。</t>
+          <t>・記録の修正は「打刻」シートを直接書き換え、「備考」に理由を書いてください。</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>・記録の修正は「打刻」シートを直接書き換え、「備考」に理由を書いてください。職員はこのファイルを見られません。</t>
+          <t>・このファイルは誰にも共有しないでください。職員は自分の分も含めて見られません。</t>
         </is>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="D6:D15">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F6:F15">
-    <cfRule type="cellIs" priority="2" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -855,10 +799,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
@@ -867,12 +811,8 @@
     <col width="7" customWidth="1" min="7" max="7"/>
     <col width="6" customWidth="1" min="8" max="8"/>
     <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="7" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="36" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="24" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -923,35 +863,16 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>場所</t>
+          <t>記録日時</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>緯度</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>経度</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>住所</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>記録日時</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
           <t>備考</t>
         </is>
       </c>
     </row>
+    <row r="2"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>